<commit_message>
Sync review data 2026-10-16
</commit_message>
<xml_diff>
--- a/review-results/复盘信息抓取-20261016.xlsx
+++ b/review-results/复盘信息抓取-20261016.xlsx
@@ -1112,1046 +1112,3926 @@
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>00:15</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>355.48</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>433.51</v>
+      </c>
       <c r="I2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>00:15</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>280.88</v>
+      </c>
       <c r="S2" s="3" t="n"/>
       <c r="T2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>355.48</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>474.79</v>
+      </c>
       <c r="I3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>280.88</v>
+      </c>
       <c r="S3" s="3" t="n"/>
       <c r="T3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>00:45</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>355.48</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>465</v>
+      </c>
       <c r="I4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>00:45</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>280.88</v>
+      </c>
       <c r="S4" s="3" t="n"/>
       <c r="T4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>355.48</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>464.8</v>
+      </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
+      <c r="L5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>280.88</v>
+      </c>
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>01:15</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>369.51</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>445</v>
+      </c>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
+      <c r="L6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>01:15</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>244</v>
+      </c>
       <c r="S6" s="3" t="n"/>
       <c r="T6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>01:30</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>369.51</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>441.51</v>
+      </c>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
+      <c r="L7" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>01:30</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>244</v>
+      </c>
       <c r="S7" s="3" t="n"/>
       <c r="T7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>01:45</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>369.51</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>430.36</v>
+      </c>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
+      <c r="L8" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>01:45</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>244</v>
+      </c>
       <c r="S8" s="3" t="n"/>
       <c r="T8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>369.35</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>431.57</v>
+      </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
+      <c r="L9" t="n">
+        <v>8</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>244</v>
+      </c>
       <c r="S9" s="3" t="n"/>
       <c r="T9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>474.23</v>
+      </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
+      <c r="L10" t="n">
+        <v>9</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S10" s="3" t="n"/>
       <c r="T10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>465</v>
+      </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
+      <c r="L11" t="n">
+        <v>10</v>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S11" s="3" t="n"/>
       <c r="T11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>02:45</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>433.73</v>
+      </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
+      <c r="L12" t="n">
+        <v>11</v>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>02:45</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S12" s="3" t="n"/>
       <c r="T12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>429.32</v>
+      </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
+      <c r="L13" t="n">
+        <v>12</v>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S13" s="3" t="n"/>
       <c r="T13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>03:15</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>415.25</v>
+      </c>
       <c r="I14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
+      <c r="L14" t="n">
+        <v>13</v>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>03:15</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S14" s="3" t="n"/>
       <c r="T14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>413.35</v>
+      </c>
       <c r="I15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="O15" s="3" t="n"/>
+      <c r="L15" t="n">
+        <v>14</v>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S15" s="3" t="n"/>
       <c r="T15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>03:45</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>410.67</v>
+      </c>
       <c r="I16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
+      <c r="L16" t="n">
+        <v>15</v>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>03:45</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S16" s="3" t="n"/>
       <c r="T16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>415.25</v>
+      </c>
       <c r="I17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="O17" s="3" t="n"/>
+      <c r="L17" t="n">
+        <v>16</v>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S17" s="3" t="n"/>
       <c r="T17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>434.47</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>410.89</v>
+      </c>
       <c r="I18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="O18" s="3" t="n"/>
+      <c r="L18" t="n">
+        <v>17</v>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S18" s="3" t="n"/>
       <c r="T18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>434.47</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>411.83</v>
+      </c>
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="O19" s="3" t="n"/>
+      <c r="L19" t="n">
+        <v>18</v>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S19" s="3" t="n"/>
       <c r="T19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>434.47</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>410</v>
+      </c>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="O20" s="3" t="n"/>
+      <c r="L20" t="n">
+        <v>19</v>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S20" s="3" t="n"/>
       <c r="T20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>434.47</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>390.38</v>
+      </c>
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="O21" s="3" t="n"/>
+      <c r="L21" t="n">
+        <v>20</v>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S21" s="3" t="n"/>
       <c r="T21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>05:15</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>446.76</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>370</v>
+      </c>
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
+      <c r="L22" t="n">
+        <v>21</v>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>05:15</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>360.85</v>
+      </c>
       <c r="S22" s="3" t="n"/>
       <c r="T22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>446.76</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>358.07</v>
+      </c>
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="O23" s="3" t="n"/>
+      <c r="L23" t="n">
+        <v>22</v>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>360.85</v>
+      </c>
       <c r="S23" s="3" t="n"/>
       <c r="T23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>446.76</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>353.54</v>
+      </c>
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="O24" s="3" t="n"/>
+      <c r="L24" t="n">
+        <v>23</v>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>360.85</v>
+      </c>
       <c r="S24" s="3" t="n"/>
       <c r="T24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>446.76</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>355.48</v>
+      </c>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="O25" s="3" t="n"/>
+      <c r="L25" t="n">
+        <v>24</v>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>360.85</v>
+      </c>
       <c r="S25" s="3" t="n"/>
       <c r="T25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>470</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>335.98</v>
+      </c>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
+      <c r="L26" t="n">
+        <v>25</v>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>361.77</v>
+      </c>
       <c r="S26" s="3" t="n"/>
       <c r="T26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>470</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>350.91</v>
+      </c>
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="O27" s="3" t="n"/>
+      <c r="L27" t="n">
+        <v>26</v>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>361.77</v>
+      </c>
       <c r="S27" s="3" t="n"/>
       <c r="T27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>470</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>414.04</v>
+      </c>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="O28" s="3" t="n"/>
+      <c r="L28" t="n">
+        <v>27</v>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>361.77</v>
+      </c>
       <c r="S28" s="3" t="n"/>
       <c r="T28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>470</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>430.14</v>
+      </c>
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="O29" s="3" t="n"/>
+      <c r="L29" t="n">
+        <v>28</v>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>361.77</v>
+      </c>
       <c r="S29" s="3" t="n"/>
       <c r="T29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>445</v>
+      </c>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="O30" s="3" t="n"/>
+      <c r="L30" t="n">
+        <v>29</v>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S30" s="3" t="n"/>
       <c r="T30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>434.35</v>
+      </c>
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
-      <c r="M31" s="3" t="n"/>
-      <c r="O31" s="3" t="n"/>
+      <c r="L31" t="n">
+        <v>30</v>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S31" s="3" t="n"/>
       <c r="T31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>425.45</v>
+      </c>
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
-      <c r="M32" s="3" t="n"/>
-      <c r="O32" s="3" t="n"/>
+      <c r="L32" t="n">
+        <v>31</v>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S32" s="3" t="n"/>
       <c r="T32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>409.66</v>
+      </c>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
-      <c r="M33" s="3" t="n"/>
-      <c r="O33" s="3" t="n"/>
+      <c r="L33" t="n">
+        <v>32</v>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="n">
+        <v>364.26</v>
+      </c>
       <c r="S33" s="3" t="n"/>
       <c r="T33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>415.25</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>395.97</v>
+      </c>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
-      <c r="M34" s="3" t="n"/>
-      <c r="O34" s="3" t="n"/>
+      <c r="L34" t="n">
+        <v>33</v>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S34" s="3" t="n"/>
       <c r="T34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>415.25</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>353.51</v>
+      </c>
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
-      <c r="M35" s="3" t="n"/>
-      <c r="O35" s="3" t="n"/>
+      <c r="L35" t="n">
+        <v>34</v>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S35" s="3" t="n"/>
       <c r="T35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>415.25</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>350.26</v>
+      </c>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
-      <c r="M36" s="3" t="n"/>
-      <c r="O36" s="3" t="n"/>
+      <c r="L36" t="n">
+        <v>35</v>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S36" s="3" t="n"/>
       <c r="T36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>415.25</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>276.08</v>
+      </c>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
-      <c r="M37" s="3" t="n"/>
-      <c r="O37" s="3" t="n"/>
+      <c r="L37" t="n">
+        <v>36</v>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S37" s="3" t="n"/>
       <c r="T37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="3" t="n"/>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>186.94</v>
+      </c>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
-      <c r="M38" s="3" t="n"/>
-      <c r="O38" s="3" t="n"/>
+      <c r="L38" t="n">
+        <v>37</v>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="n">
+        <v>320</v>
+      </c>
       <c r="S38" s="3" t="n"/>
       <c r="T38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>182.88</v>
+      </c>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
-      <c r="M39" s="3" t="n"/>
-      <c r="O39" s="3" t="n"/>
+      <c r="L39" t="n">
+        <v>38</v>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="O39" s="3" t="n">
+        <v>360.85</v>
+      </c>
       <c r="S39" s="3" t="n"/>
       <c r="T39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>184.11</v>
+      </c>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
-      <c r="M40" s="3" t="n"/>
-      <c r="O40" s="3" t="n"/>
+      <c r="L40" t="n">
+        <v>39</v>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="O40" s="3" t="n">
+        <v>320</v>
+      </c>
       <c r="S40" s="3" t="n"/>
       <c r="T40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>177.47</v>
+      </c>
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
-      <c r="M41" s="3" t="n"/>
-      <c r="O41" s="3" t="n"/>
+      <c r="L41" t="n">
+        <v>40</v>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="n">
+        <v>320</v>
+      </c>
       <c r="S41" s="3" t="n"/>
       <c r="T41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>178.71</v>
+      </c>
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
-      <c r="M42" s="3" t="n"/>
-      <c r="O42" s="3" t="n"/>
+      <c r="L42" t="n">
+        <v>41</v>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="O42" s="3" t="n">
+        <v>360.85</v>
+      </c>
       <c r="S42" s="3" t="n"/>
       <c r="T42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>175.52</v>
+      </c>
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
-      <c r="M43" s="3" t="n"/>
-      <c r="O43" s="3" t="n"/>
+      <c r="L43" t="n">
+        <v>42</v>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="n">
+        <v>361.77</v>
+      </c>
       <c r="S43" s="3" t="n"/>
       <c r="T43" s="3" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="3" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>172.96</v>
+      </c>
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
-      <c r="M44" s="3" t="n"/>
-      <c r="O44" s="3" t="n"/>
+      <c r="L44" t="n">
+        <v>43</v>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="O44" s="3" t="n">
+        <v>360.85</v>
+      </c>
       <c r="S44" s="3" t="n"/>
       <c r="T44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="3" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>186.94</v>
+      </c>
       <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
-      <c r="M45" s="3" t="n"/>
-      <c r="O45" s="3" t="n"/>
+      <c r="L45" t="n">
+        <v>44</v>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="O45" s="3" t="n">
+        <v>360.85</v>
+      </c>
       <c r="S45" s="3" t="n"/>
       <c r="T45" s="3" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="3" t="n"/>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>210</v>
+      </c>
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
-      <c r="M46" s="3" t="n"/>
-      <c r="O46" s="3" t="n"/>
+      <c r="L46" t="n">
+        <v>45</v>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="O46" s="3" t="n">
+        <v>433.32</v>
+      </c>
       <c r="S46" s="3" t="n"/>
       <c r="T46" s="3" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="3" t="n"/>
-      <c r="D47" s="3" t="n"/>
-      <c r="E47" s="3" t="n"/>
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>274.6</v>
+      </c>
       <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
-      <c r="M47" s="3" t="n"/>
-      <c r="O47" s="3" t="n"/>
+      <c r="L47" t="n">
+        <v>46</v>
+      </c>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="O47" s="3" t="n">
+        <v>433.32</v>
+      </c>
       <c r="S47" s="3" t="n"/>
       <c r="T47" s="3" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="3" t="n"/>
-      <c r="D48" s="3" t="n"/>
-      <c r="E48" s="3" t="n"/>
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>210</v>
+      </c>
       <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
-      <c r="M48" s="3" t="n"/>
-      <c r="O48" s="3" t="n"/>
+      <c r="L48" t="n">
+        <v>47</v>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="O48" s="3" t="n">
+        <v>433.32</v>
+      </c>
       <c r="S48" s="3" t="n"/>
       <c r="T48" s="3" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="3" t="n"/>
-      <c r="D49" s="3" t="n"/>
-      <c r="E49" s="3" t="n"/>
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>204.16</v>
+      </c>
       <c r="H49" s="3" t="n"/>
       <c r="I49" s="3" t="n"/>
-      <c r="M49" s="3" t="n"/>
-      <c r="O49" s="3" t="n"/>
+      <c r="L49" t="n">
+        <v>48</v>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="O49" s="3" t="n">
+        <v>433.32</v>
+      </c>
       <c r="S49" s="3" t="n"/>
       <c r="T49" s="3" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="3" t="n"/>
-      <c r="D50" s="3" t="n"/>
-      <c r="E50" s="3" t="n"/>
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>149.52</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>200.77</v>
+      </c>
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
-      <c r="M50" s="3" t="n"/>
-      <c r="O50" s="3" t="n"/>
+      <c r="L50" t="n">
+        <v>49</v>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="O50" s="3" t="n">
+        <v>433.32</v>
+      </c>
       <c r="S50" s="3" t="n"/>
       <c r="T50" s="3" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="3" t="n"/>
-      <c r="D51" s="3" t="n"/>
-      <c r="E51" s="3" t="n"/>
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>149.52</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>186.94</v>
+      </c>
       <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
-      <c r="M51" s="3" t="n"/>
-      <c r="O51" s="3" t="n"/>
+      <c r="L51" t="n">
+        <v>50</v>
+      </c>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="O51" s="3" t="n">
+        <v>433.32</v>
+      </c>
       <c r="S51" s="3" t="n"/>
       <c r="T51" s="3" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="3" t="n"/>
-      <c r="D52" s="3" t="n"/>
-      <c r="E52" s="3" t="n"/>
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>149.52</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>206.47</v>
+      </c>
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
-      <c r="M52" s="3" t="n"/>
-      <c r="O52" s="3" t="n"/>
+      <c r="L52" t="n">
+        <v>51</v>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="n">
+        <v>433.32</v>
+      </c>
       <c r="S52" s="3" t="n"/>
       <c r="T52" s="3" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="3" t="n"/>
-      <c r="D53" s="3" t="n"/>
-      <c r="E53" s="3" t="n"/>
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>149.52</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>200.57</v>
+      </c>
       <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="n"/>
-      <c r="M53" s="3" t="n"/>
-      <c r="O53" s="3" t="n"/>
+      <c r="L53" t="n">
+        <v>52</v>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="O53" s="3" t="n">
+        <v>433.32</v>
+      </c>
       <c r="S53" s="3" t="n"/>
       <c r="T53" s="3" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="3" t="n"/>
-      <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="n"/>
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>207.16</v>
+      </c>
       <c r="H54" s="3" t="n"/>
       <c r="I54" s="3" t="n"/>
-      <c r="M54" s="3" t="n"/>
-      <c r="O54" s="3" t="n"/>
+      <c r="L54" t="n">
+        <v>53</v>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="O54" s="3" t="n">
+        <v>415.23</v>
+      </c>
       <c r="S54" s="3" t="n"/>
       <c r="T54" s="3" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="3" t="n"/>
-      <c r="D55" s="3" t="n"/>
-      <c r="E55" s="3" t="n"/>
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>244.52</v>
+      </c>
       <c r="H55" s="3" t="n"/>
       <c r="I55" s="3" t="n"/>
-      <c r="M55" s="3" t="n"/>
-      <c r="O55" s="3" t="n"/>
+      <c r="L55" t="n">
+        <v>54</v>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="O55" s="3" t="n">
+        <v>415.23</v>
+      </c>
       <c r="S55" s="3" t="n"/>
       <c r="T55" s="3" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="3" t="n"/>
-      <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="n"/>
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>279.92</v>
+      </c>
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
-      <c r="M56" s="3" t="n"/>
-      <c r="O56" s="3" t="n"/>
+      <c r="L56" t="n">
+        <v>55</v>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="O56" s="3" t="n">
+        <v>415.23</v>
+      </c>
       <c r="S56" s="3" t="n"/>
       <c r="T56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="3" t="n"/>
-      <c r="D57" s="3" t="n"/>
-      <c r="E57" s="3" t="n"/>
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>234.16</v>
+      </c>
       <c r="H57" s="3" t="n"/>
       <c r="I57" s="3" t="n"/>
-      <c r="M57" s="3" t="n"/>
-      <c r="O57" s="3" t="n"/>
+      <c r="L57" t="n">
+        <v>56</v>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="O57" s="3" t="n">
+        <v>415.23</v>
+      </c>
       <c r="S57" s="3" t="n"/>
       <c r="T57" s="3" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="3" t="n"/>
-      <c r="D58" s="3" t="n"/>
-      <c r="E58" s="3" t="n"/>
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>369.51</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>279.07</v>
+      </c>
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="n"/>
-      <c r="M58" s="3" t="n"/>
-      <c r="O58" s="3" t="n"/>
+      <c r="L58" t="n">
+        <v>57</v>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S58" s="3" t="n"/>
       <c r="T58" s="3" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="3" t="n"/>
-      <c r="D59" s="3" t="n"/>
-      <c r="E59" s="3" t="n"/>
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>369.35</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>310.42</v>
+      </c>
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="3" t="n"/>
-      <c r="M59" s="3" t="n"/>
-      <c r="O59" s="3" t="n"/>
+      <c r="L59" t="n">
+        <v>58</v>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="O59" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S59" s="3" t="n"/>
       <c r="T59" s="3" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="3" t="n"/>
-      <c r="D60" s="3" t="n"/>
-      <c r="E60" s="3" t="n"/>
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>369.35</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>350.29</v>
+      </c>
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="n"/>
-      <c r="M60" s="3" t="n"/>
-      <c r="O60" s="3" t="n"/>
+      <c r="L60" t="n">
+        <v>59</v>
+      </c>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="O60" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S60" s="3" t="n"/>
       <c r="T60" s="3" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" s="3" t="n"/>
-      <c r="D61" s="3" t="n"/>
-      <c r="E61" s="3" t="n"/>
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>369.35</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>380.95</v>
+      </c>
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="n"/>
-      <c r="M61" s="3" t="n"/>
-      <c r="O61" s="3" t="n"/>
+      <c r="L61" t="n">
+        <v>60</v>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="O61" s="3" t="n">
+        <v>410.82</v>
+      </c>
       <c r="S61" s="3" t="n"/>
       <c r="T61" s="3" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" s="3" t="n"/>
-      <c r="D62" s="3" t="n"/>
-      <c r="E62" s="3" t="n"/>
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>402.8</v>
+      </c>
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="n"/>
-      <c r="M62" s="3" t="n"/>
-      <c r="O62" s="3" t="n"/>
+      <c r="L62" t="n">
+        <v>61</v>
+      </c>
+      <c r="M62" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="O62" s="3" t="n">
+        <v>480.76</v>
+      </c>
       <c r="S62" s="3" t="n"/>
       <c r="T62" s="3" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" s="3" t="n"/>
-      <c r="D63" s="3" t="n"/>
-      <c r="E63" s="3" t="n"/>
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>415.25</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>419.7</v>
+      </c>
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="n"/>
-      <c r="M63" s="3" t="n"/>
-      <c r="O63" s="3" t="n"/>
+      <c r="L63" t="n">
+        <v>62</v>
+      </c>
+      <c r="M63" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="O63" s="3" t="n">
+        <v>480.76</v>
+      </c>
       <c r="S63" s="3" t="n"/>
       <c r="T63" s="3" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" s="3" t="n"/>
-      <c r="D64" s="3" t="n"/>
-      <c r="E64" s="3" t="n"/>
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>449.48</v>
+      </c>
       <c r="H64" s="3" t="n"/>
       <c r="I64" s="3" t="n"/>
-      <c r="M64" s="3" t="n"/>
-      <c r="O64" s="3" t="n"/>
+      <c r="L64" t="n">
+        <v>63</v>
+      </c>
+      <c r="M64" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="O64" s="3" t="n">
+        <v>480.76</v>
+      </c>
       <c r="S64" s="3" t="n"/>
       <c r="T64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" s="3" t="n"/>
-      <c r="D65" s="3" t="n"/>
-      <c r="E65" s="3" t="n"/>
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>434.2</v>
+      </c>
       <c r="H65" s="3" t="n"/>
       <c r="I65" s="3" t="n"/>
-      <c r="M65" s="3" t="n"/>
-      <c r="O65" s="3" t="n"/>
+      <c r="L65" t="n">
+        <v>64</v>
+      </c>
+      <c r="M65" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="O65" s="3" t="n">
+        <v>480.76</v>
+      </c>
       <c r="S65" s="3" t="n"/>
       <c r="T65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>390.94</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>453.39</v>
+      </c>
       <c r="H66" s="3" t="n"/>
       <c r="I66" s="3" t="n"/>
-      <c r="M66" s="3" t="n"/>
-      <c r="O66" s="3" t="n"/>
+      <c r="L66" t="n">
+        <v>65</v>
+      </c>
+      <c r="M66" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="O66" s="3" t="n">
+        <v>410.48</v>
+      </c>
       <c r="S66" s="3" t="n"/>
       <c r="T66" s="3" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" s="3" t="n"/>
-      <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="n"/>
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>445.91</v>
+      </c>
       <c r="H67" s="3" t="n"/>
       <c r="I67" s="3" t="n"/>
-      <c r="M67" s="3" t="n"/>
-      <c r="O67" s="3" t="n"/>
+      <c r="L67" t="n">
+        <v>66</v>
+      </c>
+      <c r="M67" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="O67" s="3" t="n">
+        <v>410.48</v>
+      </c>
       <c r="S67" s="3" t="n"/>
       <c r="T67" s="3" t="n"/>
     </row>
     <row r="68">
-      <c r="B68" s="3" t="n"/>
-      <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>460</v>
+      </c>
       <c r="H68" s="3" t="n"/>
       <c r="I68" s="3" t="n"/>
-      <c r="M68" s="3" t="n"/>
-      <c r="O68" s="3" t="n"/>
+      <c r="L68" t="n">
+        <v>67</v>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="O68" s="3" t="n">
+        <v>410.48</v>
+      </c>
       <c r="S68" s="3" t="n"/>
       <c r="T68" s="3" t="n"/>
     </row>
     <row r="69">
-      <c r="B69" s="3" t="n"/>
-      <c r="D69" s="3" t="n"/>
-      <c r="E69" s="3" t="n"/>
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>390.54</v>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="H69" s="3" t="n"/>
       <c r="I69" s="3" t="n"/>
-      <c r="M69" s="3" t="n"/>
-      <c r="O69" s="3" t="n"/>
+      <c r="L69" t="n">
+        <v>68</v>
+      </c>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="O69" s="3" t="n">
+        <v>410.48</v>
+      </c>
       <c r="S69" s="3" t="n"/>
       <c r="T69" s="3" t="n"/>
     </row>
     <row r="70">
-      <c r="B70" s="3" t="n"/>
-      <c r="D70" s="3" t="n"/>
-      <c r="E70" s="3" t="n"/>
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>435.04</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>413.82</v>
+      </c>
       <c r="H70" s="3" t="n"/>
       <c r="I70" s="3" t="n"/>
-      <c r="M70" s="3" t="n"/>
-      <c r="O70" s="3" t="n"/>
+      <c r="L70" t="n">
+        <v>69</v>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="O70" s="3" t="n">
+        <v>181.91</v>
+      </c>
       <c r="S70" s="3" t="n"/>
       <c r="T70" s="3" t="n"/>
     </row>
     <row r="71">
-      <c r="B71" s="3" t="n"/>
-      <c r="D71" s="3" t="n"/>
-      <c r="E71" s="3" t="n"/>
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>435.04</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>413.35</v>
+      </c>
       <c r="H71" s="3" t="n"/>
       <c r="I71" s="3" t="n"/>
-      <c r="M71" s="3" t="n"/>
-      <c r="O71" s="3" t="n"/>
+      <c r="L71" t="n">
+        <v>70</v>
+      </c>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="O71" s="3" t="n">
+        <v>181.91</v>
+      </c>
       <c r="S71" s="3" t="n"/>
       <c r="T71" s="3" t="n"/>
     </row>
     <row r="72">
-      <c r="B72" s="3" t="n"/>
-      <c r="D72" s="3" t="n"/>
-      <c r="E72" s="3" t="n"/>
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>435.04</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>411.01</v>
+      </c>
       <c r="H72" s="3" t="n"/>
       <c r="I72" s="3" t="n"/>
-      <c r="M72" s="3" t="n"/>
-      <c r="O72" s="3" t="n"/>
+      <c r="L72" t="n">
+        <v>71</v>
+      </c>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="O72" s="3" t="n">
+        <v>181.91</v>
+      </c>
       <c r="S72" s="3" t="n"/>
       <c r="T72" s="3" t="n"/>
     </row>
     <row r="73">
-      <c r="B73" s="3" t="n"/>
-      <c r="D73" s="3" t="n"/>
-      <c r="E73" s="3" t="n"/>
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>435.04</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>390.38</v>
+      </c>
       <c r="H73" s="3" t="n"/>
       <c r="I73" s="3" t="n"/>
-      <c r="M73" s="3" t="n"/>
-      <c r="O73" s="3" t="n"/>
+      <c r="L73" t="n">
+        <v>72</v>
+      </c>
+      <c r="M73" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="O73" s="3" t="n">
+        <v>181.91</v>
+      </c>
       <c r="S73" s="3" t="n"/>
       <c r="T73" s="3" t="n"/>
     </row>
     <row r="74">
-      <c r="B74" s="3" t="n"/>
-      <c r="D74" s="3" t="n"/>
-      <c r="E74" s="3" t="n"/>
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>369.51</v>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>385.45</v>
+      </c>
       <c r="H74" s="3" t="n"/>
       <c r="I74" s="3" t="n"/>
-      <c r="M74" s="3" t="n"/>
-      <c r="O74" s="3" t="n"/>
+      <c r="L74" t="n">
+        <v>73</v>
+      </c>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="O74" s="3" t="n">
+        <v>244</v>
+      </c>
       <c r="S74" s="3" t="n"/>
       <c r="T74" s="3" t="n"/>
     </row>
     <row r="75">
-      <c r="B75" s="3" t="n"/>
-      <c r="D75" s="3" t="n"/>
-      <c r="E75" s="3" t="n"/>
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>369.51</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>358.07</v>
+      </c>
       <c r="H75" s="3" t="n"/>
       <c r="I75" s="3" t="n"/>
-      <c r="M75" s="3" t="n"/>
-      <c r="O75" s="3" t="n"/>
+      <c r="L75" t="n">
+        <v>74</v>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="O75" s="3" t="n">
+        <v>244</v>
+      </c>
       <c r="S75" s="3" t="n"/>
       <c r="T75" s="3" t="n"/>
     </row>
     <row r="76">
-      <c r="B76" s="3" t="n"/>
-      <c r="D76" s="3" t="n"/>
-      <c r="E76" s="3" t="n"/>
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>369.51</v>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>355.73</v>
+      </c>
       <c r="H76" s="3" t="n"/>
       <c r="I76" s="3" t="n"/>
-      <c r="M76" s="3" t="n"/>
-      <c r="O76" s="3" t="n"/>
+      <c r="L76" t="n">
+        <v>75</v>
+      </c>
+      <c r="M76" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="O76" s="3" t="n">
+        <v>244</v>
+      </c>
       <c r="S76" s="3" t="n"/>
       <c r="T76" s="3" t="n"/>
     </row>
     <row r="77">
-      <c r="B77" s="3" t="n"/>
-      <c r="D77" s="3" t="n"/>
-      <c r="E77" s="3" t="n"/>
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>369.51</v>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>345</v>
+      </c>
       <c r="H77" s="3" t="n"/>
       <c r="I77" s="3" t="n"/>
-      <c r="M77" s="3" t="n"/>
-      <c r="O77" s="3" t="n"/>
+      <c r="L77" t="n">
+        <v>76</v>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="O77" s="3" t="n">
+        <v>244</v>
+      </c>
       <c r="S77" s="3" t="n"/>
       <c r="T77" s="3" t="n"/>
     </row>
     <row r="78">
-      <c r="B78" s="3" t="n"/>
-      <c r="D78" s="3" t="n"/>
-      <c r="E78" s="3" t="n"/>
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>330.79</v>
+      </c>
       <c r="H78" s="3" t="n"/>
       <c r="I78" s="3" t="n"/>
-      <c r="M78" s="3" t="n"/>
-      <c r="O78" s="3" t="n"/>
+      <c r="L78" t="n">
+        <v>77</v>
+      </c>
+      <c r="M78" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="O78" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S78" s="3" t="n"/>
       <c r="T78" s="3" t="n"/>
     </row>
     <row r="79">
-      <c r="B79" s="3" t="n"/>
-      <c r="D79" s="3" t="n"/>
-      <c r="E79" s="3" t="n"/>
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>275.26</v>
+      </c>
       <c r="H79" s="3" t="n"/>
       <c r="I79" s="3" t="n"/>
-      <c r="M79" s="3" t="n"/>
-      <c r="O79" s="3" t="n"/>
+      <c r="L79" t="n">
+        <v>78</v>
+      </c>
+      <c r="M79" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="O79" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S79" s="3" t="n"/>
       <c r="T79" s="3" t="n"/>
     </row>
     <row r="80">
-      <c r="B80" s="3" t="n"/>
-      <c r="D80" s="3" t="n"/>
-      <c r="E80" s="3" t="n"/>
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="E80" s="3" t="n">
+        <v>282.13</v>
+      </c>
       <c r="H80" s="3" t="n"/>
       <c r="I80" s="3" t="n"/>
-      <c r="M80" s="3" t="n"/>
-      <c r="O80" s="3" t="n"/>
+      <c r="L80" t="n">
+        <v>79</v>
+      </c>
+      <c r="M80" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="O80" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S80" s="3" t="n"/>
       <c r="T80" s="3" t="n"/>
     </row>
     <row r="81">
-      <c r="B81" s="3" t="n"/>
-      <c r="D81" s="3" t="n"/>
-      <c r="E81" s="3" t="n"/>
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="E81" s="3" t="n">
+        <v>328.38</v>
+      </c>
       <c r="H81" s="3" t="n"/>
       <c r="I81" s="3" t="n"/>
-      <c r="M81" s="3" t="n"/>
-      <c r="O81" s="3" t="n"/>
+      <c r="L81" t="n">
+        <v>80</v>
+      </c>
+      <c r="M81" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="O81" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S81" s="3" t="n"/>
       <c r="T81" s="3" t="n"/>
     </row>
     <row r="82">
-      <c r="B82" s="3" t="n"/>
-      <c r="D82" s="3" t="n"/>
-      <c r="E82" s="3" t="n"/>
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>167.11</v>
+      </c>
+      <c r="E82" s="3" t="n">
+        <v>328.38</v>
+      </c>
       <c r="H82" s="3" t="n"/>
       <c r="I82" s="3" t="n"/>
-      <c r="M82" s="3" t="n"/>
-      <c r="O82" s="3" t="n"/>
+      <c r="L82" t="n">
+        <v>81</v>
+      </c>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="O82" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S82" s="3" t="n"/>
       <c r="T82" s="3" t="n"/>
     </row>
     <row r="83">
-      <c r="B83" s="3" t="n"/>
-      <c r="D83" s="3" t="n"/>
-      <c r="E83" s="3" t="n"/>
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>167.11</v>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>353.54</v>
+      </c>
       <c r="H83" s="3" t="n"/>
       <c r="I83" s="3" t="n"/>
-      <c r="M83" s="3" t="n"/>
-      <c r="O83" s="3" t="n"/>
+      <c r="L83" t="n">
+        <v>82</v>
+      </c>
+      <c r="M83" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="O83" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S83" s="3" t="n"/>
       <c r="T83" s="3" t="n"/>
     </row>
     <row r="84">
-      <c r="B84" s="3" t="n"/>
-      <c r="D84" s="3" t="n"/>
-      <c r="E84" s="3" t="n"/>
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>167.11</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>354.69</v>
+      </c>
       <c r="H84" s="3" t="n"/>
       <c r="I84" s="3" t="n"/>
-      <c r="M84" s="3" t="n"/>
-      <c r="O84" s="3" t="n"/>
+      <c r="L84" t="n">
+        <v>83</v>
+      </c>
+      <c r="M84" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="O84" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S84" s="3" t="n"/>
       <c r="T84" s="3" t="n"/>
     </row>
     <row r="85">
-      <c r="B85" s="3" t="n"/>
-      <c r="D85" s="3" t="n"/>
-      <c r="E85" s="3" t="n"/>
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>167.11</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>358.07</v>
+      </c>
       <c r="H85" s="3" t="n"/>
       <c r="I85" s="3" t="n"/>
-      <c r="M85" s="3" t="n"/>
-      <c r="O85" s="3" t="n"/>
+      <c r="L85" t="n">
+        <v>84</v>
+      </c>
+      <c r="M85" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="O85" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S85" s="3" t="n"/>
       <c r="T85" s="3" t="n"/>
     </row>
     <row r="86">
-      <c r="B86" s="3" t="n"/>
-      <c r="D86" s="3" t="n"/>
-      <c r="E86" s="3" t="n"/>
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>270</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>390.54</v>
+      </c>
       <c r="H86" s="3" t="n"/>
       <c r="I86" s="3" t="n"/>
-      <c r="M86" s="3" t="n"/>
-      <c r="O86" s="3" t="n"/>
+      <c r="L86" t="n">
+        <v>85</v>
+      </c>
+      <c r="M86" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="O86" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S86" s="3" t="n"/>
       <c r="T86" s="3" t="n"/>
     </row>
     <row r="87">
-      <c r="B87" s="3" t="n"/>
-      <c r="D87" s="3" t="n"/>
-      <c r="E87" s="3" t="n"/>
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>270</v>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>362.98</v>
+      </c>
       <c r="H87" s="3" t="n"/>
       <c r="I87" s="3" t="n"/>
-      <c r="M87" s="3" t="n"/>
-      <c r="O87" s="3" t="n"/>
+      <c r="L87" t="n">
+        <v>86</v>
+      </c>
+      <c r="M87" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="O87" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S87" s="3" t="n"/>
       <c r="T87" s="3" t="n"/>
     </row>
     <row r="88">
-      <c r="B88" s="3" t="n"/>
-      <c r="D88" s="3" t="n"/>
-      <c r="E88" s="3" t="n"/>
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>270</v>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>353</v>
+      </c>
       <c r="H88" s="3" t="n"/>
       <c r="I88" s="3" t="n"/>
-      <c r="M88" s="3" t="n"/>
-      <c r="O88" s="3" t="n"/>
+      <c r="L88" t="n">
+        <v>87</v>
+      </c>
+      <c r="M88" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="O88" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S88" s="3" t="n"/>
       <c r="T88" s="3" t="n"/>
     </row>
     <row r="89">
-      <c r="B89" s="3" t="n"/>
-      <c r="D89" s="3" t="n"/>
-      <c r="E89" s="3" t="n"/>
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>270</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>310</v>
+      </c>
       <c r="H89" s="3" t="n"/>
       <c r="I89" s="3" t="n"/>
-      <c r="M89" s="3" t="n"/>
-      <c r="O89" s="3" t="n"/>
+      <c r="L89" t="n">
+        <v>88</v>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="O89" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S89" s="3" t="n"/>
       <c r="T89" s="3" t="n"/>
     </row>
     <row r="90">
-      <c r="B90" s="3" t="n"/>
-      <c r="D90" s="3" t="n"/>
-      <c r="E90" s="3" t="n"/>
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E90" s="3" t="n">
+        <v>279.92</v>
+      </c>
       <c r="H90" s="3" t="n"/>
       <c r="I90" s="3" t="n"/>
-      <c r="M90" s="3" t="n"/>
-      <c r="O90" s="3" t="n"/>
+      <c r="L90" t="n">
+        <v>89</v>
+      </c>
+      <c r="M90" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="O90" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S90" s="3" t="n"/>
       <c r="T90" s="3" t="n"/>
     </row>
     <row r="91">
-      <c r="B91" s="3" t="n"/>
-      <c r="D91" s="3" t="n"/>
-      <c r="E91" s="3" t="n"/>
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E91" s="3" t="n">
+        <v>350.29</v>
+      </c>
       <c r="H91" s="3" t="n"/>
       <c r="I91" s="3" t="n"/>
-      <c r="M91" s="3" t="n"/>
-      <c r="O91" s="3" t="n"/>
+      <c r="L91" t="n">
+        <v>90</v>
+      </c>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="O91" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S91" s="3" t="n"/>
       <c r="T91" s="3" t="n"/>
     </row>
     <row r="92">
-      <c r="B92" s="3" t="n"/>
-      <c r="D92" s="3" t="n"/>
-      <c r="E92" s="3" t="n"/>
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E92" s="3" t="n">
+        <v>335.98</v>
+      </c>
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="n"/>
-      <c r="M92" s="3" t="n"/>
-      <c r="O92" s="3" t="n"/>
+      <c r="L92" t="n">
+        <v>91</v>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="O92" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S92" s="3" t="n"/>
       <c r="T92" s="3" t="n"/>
     </row>
     <row r="93">
-      <c r="B93" s="3" t="n"/>
-      <c r="D93" s="3" t="n"/>
-      <c r="E93" s="3" t="n"/>
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>234.16</v>
+      </c>
+      <c r="E93" s="3" t="n">
+        <v>282.1</v>
+      </c>
       <c r="I93" s="3" t="n"/>
-      <c r="M93" s="3" t="n"/>
-      <c r="O93" s="3" t="n"/>
+      <c r="L93" t="n">
+        <v>92</v>
+      </c>
+      <c r="M93" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="O93" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S93" s="3" t="n"/>
       <c r="T93" s="3" t="n"/>
     </row>
     <row r="94">
-      <c r="B94" s="3" t="n"/>
-      <c r="D94" s="3" t="n"/>
-      <c r="E94" s="3" t="n"/>
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>23:15</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>155.86</v>
+      </c>
+      <c r="E94" s="3" t="n">
+        <v>310</v>
+      </c>
       <c r="I94" s="3" t="n"/>
-      <c r="M94" s="3" t="n"/>
-      <c r="O94" s="3" t="n"/>
+      <c r="L94" t="n">
+        <v>93</v>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>23:15</t>
+        </is>
+      </c>
+      <c r="O94" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S94" s="3" t="n"/>
       <c r="T94" s="3" t="n"/>
     </row>
     <row r="95">
-      <c r="B95" s="3" t="n"/>
-      <c r="D95" s="3" t="n"/>
-      <c r="E95" s="3" t="n"/>
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>155.86</v>
+      </c>
+      <c r="E95" s="3" t="n">
+        <v>287.55</v>
+      </c>
       <c r="I95" s="3" t="n"/>
-      <c r="M95" s="3" t="n"/>
-      <c r="O95" s="3" t="n"/>
+      <c r="L95" t="n">
+        <v>94</v>
+      </c>
+      <c r="M95" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="O95" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S95" s="3" t="n"/>
       <c r="T95" s="3" t="n"/>
     </row>
     <row r="96">
-      <c r="B96" s="3" t="n"/>
-      <c r="D96" s="3" t="n"/>
-      <c r="E96" s="3" t="n"/>
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>155.86</v>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>276.08</v>
+      </c>
       <c r="I96" s="3" t="n"/>
-      <c r="M96" s="3" t="n"/>
-      <c r="O96" s="3" t="n"/>
+      <c r="L96" t="n">
+        <v>95</v>
+      </c>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
+      <c r="O96" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S96" s="3" t="n"/>
       <c r="T96" s="3" t="n"/>
     </row>
     <row r="97">
-      <c r="B97" s="3" t="n"/>
-      <c r="D97" s="3" t="n"/>
-      <c r="E97" s="3" t="n"/>
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>155.86</v>
+      </c>
+      <c r="E97" s="3" t="n">
+        <v>279.44</v>
+      </c>
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="n"/>
-      <c r="M97" s="3" t="n"/>
-      <c r="O97" s="3" t="n"/>
+      <c r="L97" t="n">
+        <v>96</v>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>20261017</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="O97" s="3" t="n">
+        <v>157.94</v>
+      </c>
       <c r="S97" s="3" t="n"/>
       <c r="T97" s="3" t="n"/>
     </row>
@@ -14508,8 +17388,32 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>实时储能充电计划及电价</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>96</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>日前储能充电计划及电价</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>96</v>
+      </c>
+      <c r="C11" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>